<commit_message>
feat: per-PWR Number of PADs with parallel pad ports (schema v3)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RVNVGCctXRyJw51L4NZ8yt
</commit_message>
<xml_diff>
--- a/examples/pwr_list.xlsx
+++ b/examples/pwr_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -437,6 +437,11 @@
           <t>PWR Plane Width</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Number of PADs</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -453,6 +458,9 @@
       <c r="D2" t="n">
         <v>60</v>
       </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -468,6 +476,9 @@
       </c>
       <c r="D3" t="n">
         <v>30</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>